<commit_message>
Some modifation on folders
</commit_message>
<xml_diff>
--- a/Day-07-Pivot-Tables/Day-07-Pivot-Tables.xlsx
+++ b/Day-07-Pivot-Tables/Day-07-Pivot-Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\90_Day_Data_Analytics\Day-07-Pivot-Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B0A4AB3-9DBD-4560-AD98-F924C641F2C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C7CB500-F884-43C1-B86B-BAE95D867C9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11280" activeTab="2" xr2:uid="{0721E76F-9BB4-4A4F-AEBD-CE115CDC013E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11280" xr2:uid="{0721E76F-9BB4-4A4F-AEBD-CE115CDC013E}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Set" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId4"/>
-    <pivotCache cacheId="9" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -94,6 +94,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_ &quot;₹&quot;\ * #,##0_ ;_ &quot;₹&quot;\ * \-#,##0_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -137,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -145,7 +150,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -156,11 +160,69 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="18">
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_ &quot;₹&quot;\ * #,##0.0_ ;_ &quot;₹&quot;\ * \-#,##0.0_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="_ &quot;₹&quot;\ * #,##0_ ;_ &quot;₹&quot;\ * \-#,##0_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_ &quot;₹&quot;\ * #,##0.0_ ;_ &quot;₹&quot;\ * \-#,##0.0_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_ [$₹-4009]\ * #,##0.0_ ;_ [$₹-4009]\ * \-#,##0.0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_ [$₹-4009]\ * #,##0.0_ ;_ [$₹-4009]\ * \-#,##0.0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -276,22 +338,7 @@
           </a:sp3d>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="dk1">
-                  <a:lumMod val="75000"/>
-                  <a:lumOff val="25000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -525,7 +572,7 @@
             <c:numRef>
               <c:f>'Pivot-Table'!$B$4:$B$6</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * "-"??_ ;_ @_ </c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>130500</c:v>
@@ -608,7 +655,7 @@
         </c:scaling>
         <c:delete val="1"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="_ [$₹-4009]\ * #,##0_ ;_ [$₹-4009]\ * \-#,##0_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ " sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -813,22 +860,7 @@
           </a:sp3d>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="dk1">
-                  <a:lumMod val="75000"/>
-                  <a:lumOff val="25000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -1071,7 +1103,7 @@
             <c:numRef>
               <c:f>'Pivot-Table'!$B$12:$B$17</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>_ "₹"\ * #,##0_ ;_ "₹"\ * \-#,##0_ ;_ "₹"\ * "-"??_ ;_ @_ </c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>110000</c:v>
@@ -1163,7 +1195,7 @@
         </c:scaling>
         <c:delete val="1"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="_ &quot;₹&quot;\ * #,##0_ ;_ &quot;₹&quot;\ * \-#,##0_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ " sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2674,7 +2706,54 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{83DFDE83-F776-483B-8C49-79117D9D1F68}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1542D7E1-C4F6-4820-BD5F-B5CA6CFAB227}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{83DFDE83-F776-483B-8C49-79117D9D1F68}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A11:B17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -2747,55 +2826,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1542D7E1-C4F6-4820-BD5F-B5CA6CFAB227}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="4">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1FA1FDFA-BA03-4DC5-91BF-FF3CBE8736A8}" name="PivotTable4" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1FA1FDFA-BA03-4DC5-91BF-FF3CBE8736A8}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="A11:B17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -2854,8 +2886,13 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0" numFmtId="168"/>
   </dataFields>
+  <formats count="1">
+    <format dxfId="1">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
   <chartFormats count="1">
     <chartFormat chart="0" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
@@ -2880,7 +2917,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0382BA16-DB42-4899-8685-65E562E63FDE}" name="PivotTable3" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0382BA16-DB42-4899-8685-65E562E63FDE}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -2912,8 +2949,25 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0" numFmtId="166"/>
   </dataFields>
+  <formats count="3">
+    <format dxfId="17">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
   <chartFormats count="1">
     <chartFormat chart="0" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
@@ -3457,13 +3511,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="6"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
@@ -3471,37 +3525,37 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4">
         <v>75500</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>7000</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6">
         <v>82500</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="6"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B11" t="s">
@@ -3509,50 +3563,50 @@
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12">
         <v>55000</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13">
         <v>18000</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14">
         <v>4000</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15">
         <v>3000</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16">
         <v>2500</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17">
         <v>82500</v>
       </c>
     </row>
@@ -3571,55 +3625,55 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="6"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="8">
         <v>130500</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="8">
         <v>10000</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="8">
         <v>140500</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="6"/>
+      <c r="B9" s="5"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B11" t="s">
@@ -3627,50 +3681,50 @@
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="9">
         <v>110000</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="9">
         <v>18000</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="9">
         <v>6000</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="9">
         <v>4000</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="9">
         <v>2500</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="9">
         <v>140500</v>
       </c>
     </row>

</xml_diff>